<commit_message>
feat(cloud): Master Cloud Daily SEO & Marketing Automation Runner (214 KWs & Multi-Sheet Sync)
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_master_dataset.xlsx
+++ b/song_anh_seo_keywords_master_dataset.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Vị Trí Thứ 2 (17/08/2026)</t>
+          <t>Vị Trí Trước Đây</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vị Trí GSC Real-time (03/09/2026)</t>
+          <t>Vị Trí GSC (TB)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -439,65 +439,45 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Search Feature Rank Top</t>
+          <t>URL Đích</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>URL Đích</t>
+          <t>Lượt Tìm Kiếm (GSC Impressions)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>7D Impressions</t>
+          <t>Lượt Click (GSC Clicks)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>7D Clicks</t>
+          <t>Tỷ Lệ CTR %</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>7D CTR %</t>
+          <t>Loại Từ Khóa</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>30D Impressions</t>
+          <t>Search Intent</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>30D Clicks</t>
+          <t>Độ Ưu Tiên</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>30D CTR %</t>
+          <t>Cụm Silo</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>Loại Từ Khóa</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Search Intent</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Độ Ưu Tiên</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Cụm Silo</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
         <is>
           <t>Ngày Cập Nhật</t>
         </is>
@@ -511,82 +491,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top 12.0 (17/08/2026)</t>
+          <t>Top 12.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Top 3.0</t>
+          <t>Top 6.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tăng 9.0 Bậc (+9.0)</t>
+          <t>Tăng 6.0 Bậc (+6.0)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+          <t>80 Imp</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1,850 Imp</t>
+          <t>7 Clicks</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>142 Clicks</t>
+          <t>8.75% CTR</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7.68%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>6,920 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>485 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>7.01%</t>
+          <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Cụm 1: Mô Hình Quy Hoạch</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -598,82 +558,62 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Top 8.0 (17/08/2026)</t>
+          <t>Top 8.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Top 3.5</t>
+          <t>Top 18.1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tăng 4.5 Bậc (+4.5)</t>
+          <t>Giảm 10.1 Bậc (-10.1)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+          <t>319 Imp</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3,200 Imp</t>
+          <t>7 Clicks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>210 Clicks</t>
+          <t>2.19% CTR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6.56%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>12,400 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>780 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>6.29%</t>
+          <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Cụm 2: Mô Hình Kiến Trúc</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -685,7 +625,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Top 14.0 (17/08/2026)</t>
+          <t>Top 14.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -700,67 +640,47 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+          <t>980 Imp</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>980 Imp</t>
+          <t>54 Clicks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>54 Clicks</t>
+          <t>5.51% CTR</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3,650 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>182 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Cụm 3: Mô Hình Cao Tầng</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -772,82 +692,62 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top 16.0 (17/08/2026)</t>
+          <t>Top 16.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Top 6.0</t>
+          <t>Top 24.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tăng 10.0 Bậc (+10.0)</t>
+          <t>Giảm 8.0 Bậc (-8.0)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+          <t>29 Imp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1,120 Imp</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>68 Clicks</t>
+          <t>3.45% CTR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.07%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4,200 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>235 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>5.60%</t>
+          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -859,7 +759,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top 22.0 (17/08/2026)</t>
+          <t>Top 22.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -874,67 +774,47 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+          <t>640 Imp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>640 Imp</t>
+          <t>25 Clicks</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25 Clicks</t>
+          <t>3.91% CTR</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,350 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>82 Clicks</t>
+          <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>3.49%</t>
+          <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 3 (P3)</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Cụm 5: Mô Hình Thiết Bị</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -946,7 +826,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 18.0 (17/08/2026)</t>
+          <t>Top 18.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -961,67 +841,47 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+          <t>720 Imp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>720 Imp</t>
+          <t>38 Clicks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>38 Clicks</t>
+          <t>5.28% CTR</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5.28%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2,700 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>130 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>4.81%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +893,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1048,67 +908,47 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+          <t>530 Imp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>530 Imp</t>
+          <t>22 Clicks</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>22 Clicks</t>
+          <t>4.15% CTR</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.15%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1,980 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>75 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>3.79%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1120,7 +960,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Top 15.0 (17/08/2026)</t>
+          <t>Top 15.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1135,67 +975,47 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+          <t>1,650 Imp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1,650 Imp</t>
+          <t>118 Clicks</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>118 Clicks</t>
+          <t>7.15% CTR</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>410 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>6.72%</t>
+          <t>Cụm 1: Mô Hình Quy Hoạch</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Cụm 1: Mô Hình Quy Hoạch</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1207,82 +1027,62 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Top 10.0 (17/08/2026)</t>
+          <t>Top 10.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Top 4.5</t>
+          <t>Top 16.2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tăng 5.5 Bậc (+5.5)</t>
+          <t>Giảm 6.2 Bậc (-6.2)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+          <t>43 Imp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2,100 Imp</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>135 Clicks</t>
+          <t>2.33% CTR</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>6.43%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7,800 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>475 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>6.09%</t>
+          <t>Cụm 2: Mô Hình Kiến Trúc</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Cụm 2: Mô Hình Kiến Trúc</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1094,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Top 13.0 (17/08/2026)</t>
+          <t>Top 13.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1309,67 +1109,47 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+          <t>870 Imp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>870 Imp</t>
+          <t>46 Clicks</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>46 Clicks</t>
+          <t>5.29% CTR</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,250 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>158 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>4.86%</t>
+          <t>Cụm 3: Mô Hình Cao Tầng</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Cụm 3: Mô Hình Cao Tầng</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1381,82 +1161,62 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Top 17.0 (17/08/2026)</t>
+          <t>Top 17.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Top 6.5</t>
+          <t>Top 2.8</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tăng 10.5 Bậc (+10.5)</t>
+          <t>Tăng 14.2 Bậc (+14.2)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+          <t>28 Imp</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>940 Imp</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>52 Clicks</t>
+          <t>3.57% CTR</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5.53%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3,500 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>180 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Cụm 4: Mô Hình KCN &amp; Nhà Máy</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1228,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Top 21.0 (17/08/2026)</t>
+          <t>Top 21.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1483,67 +1243,47 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+          <t>480 Imp</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>480 Imp</t>
+          <t>18 Clicks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>18 Clicks</t>
+          <t>3.75% CTR</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.75%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,820 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>62 Clicks</t>
+          <t>Ưu Tiên 3 (P3)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>3.41%</t>
+          <t>Cụm 5: Mô Hình Thiết Bị</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 3 (P3)</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Cụm 5: Mô Hình Thiết Bị</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1555,82 +1295,62 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Top 19.0 (17/08/2026)</t>
+          <t>Top 19.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Top 7.5</t>
+          <t>Top 5.6</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Tăng 11.5 Bậc (+11.5)</t>
+          <t>Tăng 13.4 Bậc (+13.4)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+          <t>8 Imp</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>610 Imp</t>
+          <t>1 Clicks</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>29 Clicks</t>
+          <t>12.50% CTR</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2,300 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>102 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>4.43%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1362,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Top 20.0 (17/08/2026)</t>
+          <t>Top 20.0 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1657,67 +1377,47 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+          <t>590 Imp</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>590 Imp</t>
+          <t>26 Clicks</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>26 Clicks</t>
+          <t>4.41% CTR</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.41%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2,150 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>88 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4.09%</t>
+          <t>Cụm 6: Mô Hình Công Cộng</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Cụm 6: Mô Hình Công Cộng</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1429,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Top 18.5 (17/08/2026)</t>
+          <t>Top 18.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1744,67 +1444,47 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+          <t>820 Imp</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>820 Imp</t>
+          <t>45 Clicks</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>45 Clicks</t>
+          <t>5.49% CTR</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.49%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>155 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1496,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Top 19.2 (17/08/2026)</t>
+          <t>Top 19.2 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1831,67 +1511,47 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+          <t>760 Imp</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>760 Imp</t>
+          <t>38 Clicks</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>38 Clicks</t>
+          <t>5.00% CTR</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2,850 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>134 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>4.70%</t>
+          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Cụm 7: Dịch Vụ Vận Chuyển</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1563,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Top 16.4 (17/08/2026)</t>
+          <t>Top 16.4 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1918,67 +1578,47 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>❓ People Also Ask</t>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+          <t>930 Imp</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>930 Imp</t>
+          <t>58 Clicks</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>58 Clicks</t>
+          <t>6.24% CTR</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3,480 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>198 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5.69%</t>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1630,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Top 17.1 (17/08/2026)</t>
+          <t>Top 17.1 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2005,67 +1645,47 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+          <t>880 Imp</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>880 Imp</t>
+          <t>52 Clicks</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>52 Clicks</t>
+          <t>5.91% CTR</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>5.91%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3,290 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>178 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Cụm 8: Dịch Vụ Sửa Chữa</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2077,82 +1697,62 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Top 6.5 (17/08/2026)</t>
+          <t>Top 6.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Top 2.8</t>
+          <t>Top 37.4</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tăng 3.7 Bậc (+3.7)</t>
+          <t>Giảm 30.9 Bậc (-30.9)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>📌 Local Map Pack</t>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+          <t>69 Imp</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2,950 Imp</t>
+          <t>2 Clicks</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>215 Clicks</t>
+          <t>2.90% CTR</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>7.29%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>11,200 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>765 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>6.83%</t>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2164,7 +1764,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Top 8.2 (17/08/2026)</t>
+          <t>Top 8.2 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2179,67 +1779,47 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>🌟 Featured Snippet</t>
+          <t>https://mohinhkientruc.org/</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/</t>
+          <t>2,410 Imp</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2,410 Imp</t>
+          <t>168 Clicks</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>168 Clicks</t>
+          <t>6.97% CTR</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>6.97%</t>
+          <t>Từ Khóa Chính (Core Focus)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9,150 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>590 Clicks</t>
+          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>6.45%</t>
+          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Cụm 9: Định Vị Doanh Nghiệp</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2251,7 +1831,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Top 12.5 (17/08/2026)</t>
+          <t>Top 12.5 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2266,67 +1846,47 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>🖼️ Image Pack</t>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+          <t>1,780 Imp</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>1,780 Imp</t>
+          <t>121 Clicks</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>121 Clicks</t>
+          <t>6.80% CTR</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.80%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>6,650 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>425 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6.39%</t>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>
@@ -2338,7 +1898,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Top 13.8 (17/08/2026)</t>
+          <t>Top 13.8 (17/08/2026) (17/08/2026)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2353,154 +1913,47 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🔗 Organic Sitelinks</t>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+          <t>1,620 Imp</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1,620 Imp</t>
+          <t>104 Clicks</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>104 Clicks</t>
+          <t>6.42% CTR</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>Từ Khóa Phụ (Long-tail)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>6,100 Imp</t>
+          <t>Transactional B2B</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>372 Clicks</t>
+          <t>Ưu Tiên 2 (P2)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Từ Khóa Phụ (Long-tail)</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 2 (P2)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Cụm 10: Dịch Vụ Sản Xuất</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>mô hình chung cư</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Top 1.0 (17/08/2026)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Top 1.0</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0.0 Bậc (0.0)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>🖼️ Image Pack</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>https://mohinhkientruc.org/mo-hinh-chung-cu/</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>1,820 Imp</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>156 Clicks</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>8.57%</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>6,850 Imp</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>548 Clicks</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>8.00%</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Từ Khóa Chính (Core Focus)</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Transactional B2B</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Ưu Tiên 1 (P1 - Top 1-3)</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>Cụm 3: Mô Hình Cao Tầng &amp; Chung Cư</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>25/09/2026 (Mới Nhất Real-time)</t>
+          <t>20/08/2026 (Mới Nhất Real-time)</t>
         </is>
       </c>
     </row>

</xml_diff>